<commit_message>
Update dashboard data from source files
</commit_message>
<xml_diff>
--- a/Laporan_Keuangan.xlsx
+++ b/Laporan_Keuangan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dashboard_Kantin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DF7CE8A-0605-415E-84DA-0B521DD41604}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{439C7280-3FEE-455E-B9FB-2EE6A43025F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{1FEE58AC-2034-4D8B-8E5C-AA929BD445EC}"/>
   </bookViews>
@@ -275,7 +275,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -298,12 +298,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -329,10 +355,16 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -688,22 +720,22 @@
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15"/>
-      <c r="D1" s="14" t="s">
+      <c r="C1" s="16"/>
+      <c r="D1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="15"/>
-      <c r="F1" s="16" t="s">
+      <c r="E1" s="16"/>
+      <c r="F1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="15"/>
-      <c r="H1" s="16" t="s">
+      <c r="G1" s="18"/>
+      <c r="H1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="15"/>
+      <c r="I1" s="18"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
@@ -1980,6 +2012,12 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>